<commit_message>
Feed results.json into the scoring workbook
  Add a Checks sheet with the run_tests.py results and derive the
  security hard-fail flag and tool breadth on Scores from it. Fill
  Tasks from any T1-T8 results. Drop a malformed results.json entry
  and split quoted slug lists in run_tests.py. Update HANDOFF.md.

  Co-Authored-By: Claude Opus 5.5
</commit_message>
<xml_diff>
--- a/mcp-plugin-scoring.xlsx
+++ b/mcp-plugin-scoring.xlsx
@@ -10,8 +10,9 @@
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scores" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Plugins" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Weights" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Checks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Plugins" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Weights" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -145,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,7 +193,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -207,6 +208,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -613,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -643,132 +650,146 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2. On the Scores sheet, fill the yellow cells with a score from 0 to 5 (blue text = your input). Grey-header columns marked (auto) are formulas, so leave them alone.</t>
+          <t>2. On the Scores sheet, fill the yellow cells with a score from 0 to 5 (blue text = your input). Grey-header columns marked (auto) are formulas, so leave them alone. 'Breadth of tools (auto)' is yellow where there is no automated result: score those by hand.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>3. Set 'Security hard fail?' to Y for a serious security failure (no auth, everything exposed by default). The plugin's total is then capped (Weights sheet).</t>
+          <t>3. 'Security hard fail? (auto)' comes from the unauthenticated probe on the Checks sheet: Y when the enabled endpoint returns tools without credentials and the source does not show it is public by design. The plugin's total is then capped (Weights sheet).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>This workbook is regenerated from shortlist.csv and results.json (python3 build_scoring_sheet.py), so record results in results.json rather than typing them here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>4. Rank appears once both Setup and Security have at least one score. Weights, thresholds and the cap live on the Weights sheet.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Scoring scale (0-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>0 = missing or broken   1 = poor   2 = weak   3 = acceptable   4 = good   5 = excellent</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>0 = missing or broken   1 = poor   2 = weak   3 = acceptable   4 = good   5 = excellent</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Example: 'In-plugin connection guide' = 5 if the plugin shows a ready-to-copy Claude Desktop config; 3 if there is generic text only; 0 if nothing.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Colour key</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Blue text on yellow = input.   Black = formula or fixed data.   Weights and thresholds on the Weights sheet are inputs too.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Weights: area weights (must total 100), hard-fail cap, thresholds for the auto-scored columns.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Plugins: WordPress.org data for each plugin (fetched 2026-10-15), plus the mcp-adapter baseline reference row.</t>
+          <t>Weights: area weights (must total 100), hard-fail cap, thresholds for the auto-scored columns.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Scores: one row per plugin; weighted total out of 100 and rank.</t>
+          <t>Plugins: WordPress.org data for each plugin (fetched 2026-10-15), plus the mcp-adapter baseline reference row.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Tasks: the 8 standard tasks, run via Claude Desktop, per plugin.</t>
+          <t>Scores: one row per plugin; weighted total out of 100 and rank.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Tasks: the 8 standard tasks, run via Claude Desktop, per plugin. Results already in results.json are filled in.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Checks: automated results from run_tests.py (results.json): out-of-the-box state, unauthenticated probe, auth method, tool count, breadth, Abilities API use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>mcp-adapter is the official WordPress MCP Adapter. It is listed on the Plugins sheet as the reference point for comparison and is not scored or ranked.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Lanes</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>established = 100+ installs.  challenger = under 100 installs, hand-picked after a pre-screen, so newer plugins get a fair chance. Both lanes are scored identically.</t>
         </is>
@@ -964,9 +985,9 @@
           <t>Task pass rate (auto)</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
-        <is>
-          <t>Breadth of tools</t>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Breadth of tools (auto)</t>
         </is>
       </c>
       <c r="S4" s="7" t="inlineStr">
@@ -1016,7 +1037,7 @@
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>Security hard fail? (Y/N)</t>
+          <t>Security hard fail? (auto)</t>
         </is>
       </c>
       <c r="AC4" s="11" t="inlineStr">
@@ -1079,7 +1100,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B5,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B5,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R5" s="14" t="n"/>
+      <c r="R5" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B5,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S5" s="14" t="n"/>
       <c r="T5" s="15">
         <f>IF(COUNT(Q5:S5)=0,0,AVERAGE(Q5:S5)/5*Weights!$B$8)</f>
@@ -1107,7 +1131,10 @@
         <f>IF(COUNT(U5:Z5)=0,0,AVERAGE(U5:Z5)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB5" s="18" t="n"/>
+      <c r="AB5" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B5,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC5" s="19">
         <f>I5+P5+T5+AA5</f>
         <v/>
@@ -1189,7 +1216,10 @@
         <f>IF(COUNT(U6:Z6)=0,0,AVERAGE(U6:Z6)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB6" s="18" t="n"/>
+      <c r="AB6" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B6,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC6" s="19">
         <f>I6+P6+T6+AA6</f>
         <v/>
@@ -1243,7 +1273,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B7,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B7,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R7" s="14" t="n"/>
+      <c r="R7" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B7,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S7" s="14" t="n"/>
       <c r="T7" s="15">
         <f>IF(COUNT(Q7:S7)=0,0,AVERAGE(Q7:S7)/5*Weights!$B$8)</f>
@@ -1271,7 +1304,10 @@
         <f>IF(COUNT(U7:Z7)=0,0,AVERAGE(U7:Z7)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB7" s="18" t="n"/>
+      <c r="AB7" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B7,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC7" s="19">
         <f>I7+P7+T7+AA7</f>
         <v/>
@@ -1325,7 +1361,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B8,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B8,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R8" s="14" t="n"/>
+      <c r="R8" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B8,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S8" s="14" t="n"/>
       <c r="T8" s="15">
         <f>IF(COUNT(Q8:S8)=0,0,AVERAGE(Q8:S8)/5*Weights!$B$8)</f>
@@ -1353,7 +1392,10 @@
         <f>IF(COUNT(U8:Z8)=0,0,AVERAGE(U8:Z8)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB8" s="18" t="n"/>
+      <c r="AB8" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B8,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC8" s="19">
         <f>I8+P8+T8+AA8</f>
         <v/>
@@ -1435,7 +1477,10 @@
         <f>IF(COUNT(U9:Z9)=0,0,AVERAGE(U9:Z9)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB9" s="18" t="n"/>
+      <c r="AB9" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B9,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC9" s="19">
         <f>I9+P9+T9+AA9</f>
         <v/>
@@ -1489,7 +1534,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B10,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B10,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R10" s="14" t="n"/>
+      <c r="R10" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B10,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S10" s="14" t="n"/>
       <c r="T10" s="15">
         <f>IF(COUNT(Q10:S10)=0,0,AVERAGE(Q10:S10)/5*Weights!$B$8)</f>
@@ -1517,7 +1565,10 @@
         <f>IF(COUNT(U10:Z10)=0,0,AVERAGE(U10:Z10)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB10" s="18" t="n"/>
+      <c r="AB10" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B10,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC10" s="19">
         <f>I10+P10+T10+AA10</f>
         <v/>
@@ -1599,7 +1650,10 @@
         <f>IF(COUNT(U11:Z11)=0,0,AVERAGE(U11:Z11)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB11" s="18" t="n"/>
+      <c r="AB11" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B11,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC11" s="19">
         <f>I11+P11+T11+AA11</f>
         <v/>
@@ -1653,7 +1707,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B12,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B12,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R12" s="14" t="n"/>
+      <c r="R12" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B12,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S12" s="14" t="n"/>
       <c r="T12" s="15">
         <f>IF(COUNT(Q12:S12)=0,0,AVERAGE(Q12:S12)/5*Weights!$B$8)</f>
@@ -1681,7 +1738,10 @@
         <f>IF(COUNT(U12:Z12)=0,0,AVERAGE(U12:Z12)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB12" s="18" t="n"/>
+      <c r="AB12" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B12,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC12" s="19">
         <f>I12+P12+T12+AA12</f>
         <v/>
@@ -1735,7 +1795,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B13,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B13,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R13" s="14" t="n"/>
+      <c r="R13" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B13,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S13" s="14" t="n"/>
       <c r="T13" s="15">
         <f>IF(COUNT(Q13:S13)=0,0,AVERAGE(Q13:S13)/5*Weights!$B$8)</f>
@@ -1763,7 +1826,10 @@
         <f>IF(COUNT(U13:Z13)=0,0,AVERAGE(U13:Z13)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB13" s="18" t="n"/>
+      <c r="AB13" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B13,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC13" s="19">
         <f>I13+P13+T13+AA13</f>
         <v/>
@@ -1845,7 +1911,10 @@
         <f>IF(COUNT(U14:Z14)=0,0,AVERAGE(U14:Z14)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB14" s="18" t="n"/>
+      <c r="AB14" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B14,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC14" s="19">
         <f>I14+P14+T14+AA14</f>
         <v/>
@@ -1899,7 +1968,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B15,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B15,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R15" s="14" t="n"/>
+      <c r="R15" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B15,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S15" s="14" t="n"/>
       <c r="T15" s="15">
         <f>IF(COUNT(Q15:S15)=0,0,AVERAGE(Q15:S15)/5*Weights!$B$8)</f>
@@ -1927,7 +1999,10 @@
         <f>IF(COUNT(U15:Z15)=0,0,AVERAGE(U15:Z15)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB15" s="18" t="n"/>
+      <c r="AB15" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B15,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC15" s="19">
         <f>I15+P15+T15+AA15</f>
         <v/>
@@ -1981,7 +2056,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B16,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B16,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R16" s="14" t="n"/>
+      <c r="R16" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B16,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S16" s="14" t="n"/>
       <c r="T16" s="15">
         <f>IF(COUNT(Q16:S16)=0,0,AVERAGE(Q16:S16)/5*Weights!$B$8)</f>
@@ -2009,7 +2087,10 @@
         <f>IF(COUNT(U16:Z16)=0,0,AVERAGE(U16:Z16)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB16" s="18" t="n"/>
+      <c r="AB16" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B16,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC16" s="19">
         <f>I16+P16+T16+AA16</f>
         <v/>
@@ -2063,7 +2144,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B17,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B17,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R17" s="14" t="n"/>
+      <c r="R17" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B17,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S17" s="14" t="n"/>
       <c r="T17" s="15">
         <f>IF(COUNT(Q17:S17)=0,0,AVERAGE(Q17:S17)/5*Weights!$B$8)</f>
@@ -2091,7 +2175,10 @@
         <f>IF(COUNT(U17:Z17)=0,0,AVERAGE(U17:Z17)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB17" s="18" t="n"/>
+      <c r="AB17" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B17,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC17" s="19">
         <f>I17+P17+T17+AA17</f>
         <v/>
@@ -2145,7 +2232,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B18,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B18,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R18" s="14" t="n"/>
+      <c r="R18" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B18,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S18" s="14" t="n"/>
       <c r="T18" s="15">
         <f>IF(COUNT(Q18:S18)=0,0,AVERAGE(Q18:S18)/5*Weights!$B$8)</f>
@@ -2173,7 +2263,10 @@
         <f>IF(COUNT(U18:Z18)=0,0,AVERAGE(U18:Z18)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB18" s="18" t="n"/>
+      <c r="AB18" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B18,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC18" s="19">
         <f>I18+P18+T18+AA18</f>
         <v/>
@@ -2255,7 +2348,10 @@
         <f>IF(COUNT(U19:Z19)=0,0,AVERAGE(U19:Z19)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB19" s="18" t="n"/>
+      <c r="AB19" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B19,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC19" s="19">
         <f>I19+P19+T19+AA19</f>
         <v/>
@@ -2309,7 +2405,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B20,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B20,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R20" s="14" t="n"/>
+      <c r="R20" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B20,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S20" s="14" t="n"/>
       <c r="T20" s="15">
         <f>IF(COUNT(Q20:S20)=0,0,AVERAGE(Q20:S20)/5*Weights!$B$8)</f>
@@ -2337,7 +2436,10 @@
         <f>IF(COUNT(U20:Z20)=0,0,AVERAGE(U20:Z20)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB20" s="18" t="n"/>
+      <c r="AB20" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B20,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC20" s="19">
         <f>I20+P20+T20+AA20</f>
         <v/>
@@ -2419,7 +2521,10 @@
         <f>IF(COUNT(U21:Z21)=0,0,AVERAGE(U21:Z21)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB21" s="18" t="n"/>
+      <c r="AB21" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B21,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC21" s="19">
         <f>I21+P21+T21+AA21</f>
         <v/>
@@ -2501,7 +2606,10 @@
         <f>IF(COUNT(U22:Z22)=0,0,AVERAGE(U22:Z22)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB22" s="18" t="n"/>
+      <c r="AB22" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B22,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC22" s="19">
         <f>I22+P22+T22+AA22</f>
         <v/>
@@ -2583,7 +2691,10 @@
         <f>IF(COUNT(U23:Z23)=0,0,AVERAGE(U23:Z23)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB23" s="18" t="n"/>
+      <c r="AB23" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B23,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC23" s="19">
         <f>I23+P23+T23+AA23</f>
         <v/>
@@ -2637,7 +2748,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B24,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B24,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R24" s="14" t="n"/>
+      <c r="R24" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B24,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S24" s="14" t="n"/>
       <c r="T24" s="15">
         <f>IF(COUNT(Q24:S24)=0,0,AVERAGE(Q24:S24)/5*Weights!$B$8)</f>
@@ -2665,7 +2779,10 @@
         <f>IF(COUNT(U24:Z24)=0,0,AVERAGE(U24:Z24)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB24" s="18" t="n"/>
+      <c r="AB24" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B24,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC24" s="19">
         <f>I24+P24+T24+AA24</f>
         <v/>
@@ -2719,7 +2836,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B25,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B25,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R25" s="14" t="n"/>
+      <c r="R25" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B25,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S25" s="14" t="n"/>
       <c r="T25" s="15">
         <f>IF(COUNT(Q25:S25)=0,0,AVERAGE(Q25:S25)/5*Weights!$B$8)</f>
@@ -2747,7 +2867,10 @@
         <f>IF(COUNT(U25:Z25)=0,0,AVERAGE(U25:Z25)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB25" s="18" t="n"/>
+      <c r="AB25" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B25,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC25" s="19">
         <f>I25+P25+T25+AA25</f>
         <v/>
@@ -2801,7 +2924,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B26,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B26,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R26" s="14" t="n"/>
+      <c r="R26" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B26,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S26" s="14" t="n"/>
       <c r="T26" s="15">
         <f>IF(COUNT(Q26:S26)=0,0,AVERAGE(Q26:S26)/5*Weights!$B$8)</f>
@@ -2829,7 +2955,10 @@
         <f>IF(COUNT(U26:Z26)=0,0,AVERAGE(U26:Z26)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB26" s="18" t="n"/>
+      <c r="AB26" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B26,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC26" s="19">
         <f>I26+P26+T26+AA26</f>
         <v/>
@@ -2883,7 +3012,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B27,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B27,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R27" s="14" t="n"/>
+      <c r="R27" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B27,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S27" s="14" t="n"/>
       <c r="T27" s="15">
         <f>IF(COUNT(Q27:S27)=0,0,AVERAGE(Q27:S27)/5*Weights!$B$8)</f>
@@ -2911,7 +3043,10 @@
         <f>IF(COUNT(U27:Z27)=0,0,AVERAGE(U27:Z27)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB27" s="18" t="n"/>
+      <c r="AB27" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B27,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC27" s="19">
         <f>I27+P27+T27+AA27</f>
         <v/>
@@ -2993,7 +3128,10 @@
         <f>IF(COUNT(U28:Z28)=0,0,AVERAGE(U28:Z28)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB28" s="18" t="n"/>
+      <c r="AB28" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B28,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC28" s="19">
         <f>I28+P28+T28+AA28</f>
         <v/>
@@ -3075,7 +3213,10 @@
         <f>IF(COUNT(U29:Z29)=0,0,AVERAGE(U29:Z29)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB29" s="18" t="n"/>
+      <c r="AB29" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B29,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC29" s="19">
         <f>I29+P29+T29+AA29</f>
         <v/>
@@ -3129,7 +3270,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B30,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B30,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R30" s="14" t="n"/>
+      <c r="R30" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B30,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S30" s="14" t="n"/>
       <c r="T30" s="15">
         <f>IF(COUNT(Q30:S30)=0,0,AVERAGE(Q30:S30)/5*Weights!$B$8)</f>
@@ -3157,7 +3301,10 @@
         <f>IF(COUNT(U30:Z30)=0,0,AVERAGE(U30:Z30)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB30" s="18" t="n"/>
+      <c r="AB30" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B30,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC30" s="19">
         <f>I30+P30+T30+AA30</f>
         <v/>
@@ -3211,7 +3358,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B31,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B31,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R31" s="14" t="n"/>
+      <c r="R31" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B31,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S31" s="14" t="n"/>
       <c r="T31" s="15">
         <f>IF(COUNT(Q31:S31)=0,0,AVERAGE(Q31:S31)/5*Weights!$B$8)</f>
@@ -3239,7 +3389,10 @@
         <f>IF(COUNT(U31:Z31)=0,0,AVERAGE(U31:Z31)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB31" s="18" t="n"/>
+      <c r="AB31" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B31,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC31" s="19">
         <f>I31+P31+T31+AA31</f>
         <v/>
@@ -3321,7 +3474,10 @@
         <f>IF(COUNT(U32:Z32)=0,0,AVERAGE(U32:Z32)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB32" s="18" t="n"/>
+      <c r="AB32" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B32,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC32" s="19">
         <f>I32+P32+T32+AA32</f>
         <v/>
@@ -3375,7 +3531,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B33,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B33,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R33" s="14" t="n"/>
+      <c r="R33" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B33,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S33" s="14" t="n"/>
       <c r="T33" s="15">
         <f>IF(COUNT(Q33:S33)=0,0,AVERAGE(Q33:S33)/5*Weights!$B$8)</f>
@@ -3403,7 +3562,10 @@
         <f>IF(COUNT(U33:Z33)=0,0,AVERAGE(U33:Z33)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB33" s="18" t="n"/>
+      <c r="AB33" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B33,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC33" s="19">
         <f>I33+P33+T33+AA33</f>
         <v/>
@@ -3457,7 +3619,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B34,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B34,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R34" s="14" t="n"/>
+      <c r="R34" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B34,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S34" s="14" t="n"/>
       <c r="T34" s="15">
         <f>IF(COUNT(Q34:S34)=0,0,AVERAGE(Q34:S34)/5*Weights!$B$8)</f>
@@ -3485,7 +3650,10 @@
         <f>IF(COUNT(U34:Z34)=0,0,AVERAGE(U34:Z34)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB34" s="18" t="n"/>
+      <c r="AB34" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B34,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC34" s="19">
         <f>I34+P34+T34+AA34</f>
         <v/>
@@ -3539,7 +3707,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B35,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B35,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R35" s="14" t="n"/>
+      <c r="R35" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B35,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S35" s="14" t="n"/>
       <c r="T35" s="15">
         <f>IF(COUNT(Q35:S35)=0,0,AVERAGE(Q35:S35)/5*Weights!$B$8)</f>
@@ -3567,7 +3738,10 @@
         <f>IF(COUNT(U35:Z35)=0,0,AVERAGE(U35:Z35)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB35" s="18" t="n"/>
+      <c r="AB35" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B35,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC35" s="19">
         <f>I35+P35+T35+AA35</f>
         <v/>
@@ -3621,7 +3795,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B36,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B36,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R36" s="14" t="n"/>
+      <c r="R36" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B36,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S36" s="14" t="n"/>
       <c r="T36" s="15">
         <f>IF(COUNT(Q36:S36)=0,0,AVERAGE(Q36:S36)/5*Weights!$B$8)</f>
@@ -3649,7 +3826,10 @@
         <f>IF(COUNT(U36:Z36)=0,0,AVERAGE(U36:Z36)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB36" s="18" t="n"/>
+      <c r="AB36" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B36,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC36" s="19">
         <f>I36+P36+T36+AA36</f>
         <v/>
@@ -3703,7 +3883,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B37,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B37,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R37" s="14" t="n"/>
+      <c r="R37" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B37,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S37" s="14" t="n"/>
       <c r="T37" s="15">
         <f>IF(COUNT(Q37:S37)=0,0,AVERAGE(Q37:S37)/5*Weights!$B$8)</f>
@@ -3731,7 +3914,10 @@
         <f>IF(COUNT(U37:Z37)=0,0,AVERAGE(U37:Z37)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB37" s="18" t="n"/>
+      <c r="AB37" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B37,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC37" s="19">
         <f>I37+P37+T37+AA37</f>
         <v/>
@@ -3813,7 +3999,10 @@
         <f>IF(COUNT(U38:Z38)=0,0,AVERAGE(U38:Z38)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB38" s="18" t="n"/>
+      <c r="AB38" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B38,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC38" s="19">
         <f>I38+P38+T38+AA38</f>
         <v/>
@@ -3867,7 +4056,10 @@
         <f>IFERROR(IF(INDEX(Tasks!$K$5:$K$39,MATCH($B39,Tasks!$A$5:$A$39,0))="","",INDEX(Tasks!$K$5:$K$39,MATCH($B39,Tasks!$A$5:$A$39,0))*5),"")</f>
         <v/>
       </c>
-      <c r="R39" s="14" t="n"/>
+      <c r="R39" s="16">
+        <f>INDEX(Checks!$K$5:$K$39,MATCH($B39,Checks!$A$5:$A$39,0))/9*5</f>
+        <v/>
+      </c>
       <c r="S39" s="14" t="n"/>
       <c r="T39" s="15">
         <f>IF(COUNT(Q39:S39)=0,0,AVERAGE(Q39:S39)/5*Weights!$B$8)</f>
@@ -3895,7 +4087,10 @@
         <f>IF(COUNT(U39:Z39)=0,0,AVERAGE(U39:Z39)/5*Weights!$B$9)</f>
         <v/>
       </c>
-      <c r="AB39" s="18" t="n"/>
+      <c r="AB39" s="18">
+        <f>IFERROR(""&amp;INDEX(Checks!$G$5:$G$39,MATCH($B39,Checks!$A$5:$A$39,0)),"")</f>
+        <v/>
+      </c>
       <c r="AC39" s="19">
         <f>I39+P39+T39+AA39</f>
         <v/>
@@ -3916,13 +4111,10 @@
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 Y5 Y6 Y7 Y8 Y9 Y10 Y11 Y12 Y13 Y14 Y15 Y16 Y17 Y18 Y19 Y20 Y21 Y22 Y23 Y24 Y25 Y26 Y27 Y28 Y29 Y30 Y31 Y32 Y33 Y34 Y35 Y36 Y37 Y38 Y39 Z5 Z6 Z7 Z8 Z9 Z10 Z11 Z12 Z13 Z14 Z15 Z16 Z17 Z18 Z19 Z20 Z21 Z22 Z23 Z24 Z25 Z26 Z27 Z28 Z29 Z30 Z31 Z32 Z33 Z34 Z35 Z36 Z37 Z38 Z39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter a whole number from 0 to 5." type="whole" operator="between">
+  <dataValidations count="1">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 R6 R9 R11 R14 R19 R21 R22 R23 R28 R29 R32 R38 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 Y5 Y6 Y7 Y8 Y9 Y10 Y11 Y12 Y13 Y14 Y15 Y16 Y17 Y18 Y19 Y20 Y21 Y22 Y23 Y24 Y25 Y26 Y27 Y28 Y29 Y30 Y31 Y32 Y33 Y34 Y35 Y36 Y37 Y38 Y39 Z5 Z6 Z7 Z8 Z9 Z10 Z11 Z12 Z13 Z14 Z15 Z16 Z17 Z18 Z19 Z20 Z21 Z22 Z23 Z24 Z25 Z26 Z27 Z28 Z29 Z30 Z31 Z32 Z33 Z34 Z35 Z36 Z37 Z38 Z39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter a whole number from 0 to 5." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>5</formula2>
-    </dataValidation>
-    <dataValidation sqref="AB5 AB6 AB7 AB8 AB9 AB10 AB11 AB12 AB13 AB14 AB15 AB16 AB17 AB18 AB19 AB20 AB21 AB22 AB23 AB24 AB25 AB26 AB27 AB28 AB29 AB30 AB31 AB32 AB33 AB34 AB35 AB36 AB37 AB38 AB39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5035,6 +5227,2380 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Automated checks (run_tests.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>From results.json. Out of the box = before MCP is switched on; A3 = after switching it on and enabling every tool. Breadth matches tool and ability names, so it undercounts generic tools. Blank = not run or needs the manual sheet (OAuth, external server).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="54" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>MCP routes before enabling</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Out of the box (A3pre)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Unauthenticated after enabling (A3)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Hard fail (auto)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Auth method</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Abilities behind meta-tools</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Areas covered (of 9)</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Areas</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Abilities API / MCP Adapter</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>A3 detail</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>Last run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>ai-engine</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>AI Engine – The Chatbot, AI Framework &amp; MCP for WordPress</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>3.8.6</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="J5" s="24" t="inlineStr"/>
+      <c r="K5" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, users, plugins, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>reads-abilities</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O5" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>vibe-ai</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>WPVibe – MCP Server for WordPress, works with Claude, ChatGPT &amp; other AI MCP agents</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>1.20.5</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr"/>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>External (N/A)</t>
+        </is>
+      </c>
+      <c r="I6" s="24" t="inlineStr"/>
+      <c r="J6" s="24" t="inlineStr"/>
+      <c r="K6" s="24" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>MCP server runs outside WordPress. Relays MCP through the hosted wpvibe.ai service using an application password; no MCP route on the site.</t>
+        </is>
+      </c>
+      <c r="O6" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>easy-mcp-ai</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Easy MCP AI – Connect Claude to WordPress: MCP Server for ChatGPT &amp; AI Agents</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>2.2.1</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>66</v>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>131</v>
+      </c>
+      <c r="J7" s="24" t="inlineStr"/>
+      <c r="K7" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings, blocks, woocommerce</t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O7" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>royal-mcp</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Royal MCP – Secure AI Connector for Claude, ChatGPT &amp; any LLM via MCP</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>1.5.10</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>259</v>
+      </c>
+      <c r="J8" s="24" t="inlineStr"/>
+      <c r="K8" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings, blocks, woocommerce</t>
+        </is>
+      </c>
+      <c r="M8" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required. Use Authorization: Bearer &lt;token&gt; or X-Royal-MCP-API-Key header.)</t>
+        </is>
+      </c>
+      <c r="O8" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>miniorange-secure-mcp-server</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Secure MCP Server for Claude, ChatGPT, Gemini and other AI Agents</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>1.5.2</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>23</v>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="inlineStr"/>
+      <c r="J9" s="24" t="inlineStr"/>
+      <c r="K9" s="24" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="25" t="inlineStr">
+        <is>
+          <t>reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (A valid OAuth bearer token is required.)</t>
+        </is>
+      </c>
+      <c r="O9" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>wsp-mcp-ai-agents-connector</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>WSP MCP – Free MCP Plugin for WordPress: Connect Claude, ChatGPT &amp; AI Agents</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>2.9.6</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" s="24" t="inlineStr"/>
+      <c r="K10" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, blocks</t>
+        </is>
+      </c>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required. Use an Application Password (Basic), Authorization: Bearer &lt;api-key-or-oauth-token&gt;, or the X-WSP-MCP-API-Key header.)</t>
+        </is>
+      </c>
+      <c r="O10" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>cowboy-mcp</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Cowboy MCP – Free MCP Server with Undo for Claude &amp; ChatGPT</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>1.7.4</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="24" t="inlineStr"/>
+      <c r="K11" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O11" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>stifli-flex-mcp</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Flex MCP – Connect ChatGPT, Claude and AI agents with MCP, Undo, Abilities and Tools.</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>3.6.1</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="J12" s="24" t="inlineStr"/>
+      <c r="K12" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings, woocommerce</t>
+        </is>
+      </c>
+      <c r="M12" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O12" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>agent-abilities-for-mcp</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Agent Abilities for MCP – Connect Claude and ChatGPT with Permission Controls and Audit Log</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>1.9.0</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>85</v>
+      </c>
+      <c r="J13" s="24" t="inlineStr"/>
+      <c r="K13" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O13" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>diviops-agent</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>DiviOps Agent</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>1.5.46</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr"/>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>External (N/A)</t>
+        </is>
+      </c>
+      <c r="I14" s="24" t="inlineStr"/>
+      <c r="J14" s="24" t="inlineStr"/>
+      <c r="K14" s="24" t="inlineStr"/>
+      <c r="L14" s="13" t="inlineStr"/>
+      <c r="M14" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>MCP server runs outside WordPress. MCP server is the separate @diviops/mcp-server npm package; the plugin adds REST endpoints it calls with an application password.</t>
+        </is>
+      </c>
+      <c r="O14" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>ai-workflow-automation-ai-agent-hub</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>MCP Server for WordPress – Connect Claude, ChatGPT &amp; Gemini | AtlasMCP</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>1.9.3</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>57</v>
+      </c>
+      <c r="J15" s="24" t="inlineStr"/>
+      <c r="K15" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings</t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O15" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>nibwp</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>NIBWP – Self-Hosted MCP Server – Connect Claude, ChatGPT, Cursor &amp; Any AI Agent via MCP</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>1.2.11</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" s="24" t="n">
+        <v>68</v>
+      </c>
+      <c r="K16" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, users, plugins, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O16" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>mountdev-ai-mcp-connector</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>MountDev AI MCP Connector for WordPress</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>2.2.0</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I17" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="J17" s="24" t="inlineStr"/>
+      <c r="K17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, users, settings</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>reads-abilities</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O17" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>iato-mcp</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>IATO MCP</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>1.14.0</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I18" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="J18" s="24" t="inlineStr"/>
+      <c r="K18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, settings</t>
+        </is>
+      </c>
+      <c r="M18" s="25" t="inlineStr">
+        <is>
+          <t>registers-abilities</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O18" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>siteskite</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>SiteSkite – Secure MCP &amp; AI WebOps. Connect ChatGPT, Claude, or Any AI Agent via MCP</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>2.2.11</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I19" s="24" t="inlineStr"/>
+      <c r="J19" s="24" t="inlineStr"/>
+      <c r="K19" s="24" t="inlineStr"/>
+      <c r="L19" s="13" t="inlineStr"/>
+      <c r="M19" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required. Connect this app with OAuth, or use a WordPress Application Password with Basic auth.)</t>
+        </is>
+      </c>
+      <c r="O19" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>invizo-mcp</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Invizo MCP – Secure AI Connector for Claude, Codex, Cursor and WooCommerce</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>2.0.8</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="24" t="n">
+        <v>91</v>
+      </c>
+      <c r="K20" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M20" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O20" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>ylabs-ai-assistant-connector</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>YLabs AI Assistant Connector</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>0.9.14</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr"/>
+      <c r="H21" s="24" t="inlineStr">
+        <is>
+          <t>External (N/A)</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="inlineStr"/>
+      <c r="J21" s="24" t="inlineStr"/>
+      <c r="K21" s="24" t="inlineStr"/>
+      <c r="L21" s="13" t="inlineStr"/>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>MCP server runs outside WordPress. Adds wp-agent/v1 REST endpoints for an external assistant that authenticates with application passwords; no MCP endpoint on the site.</t>
+        </is>
+      </c>
+      <c r="O21" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>albert-ai-butler</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Albert – Connect AI Assistants to WordPress</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>1.5.0</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="inlineStr"/>
+      <c r="J22" s="24" t="inlineStr"/>
+      <c r="K22" s="24" t="inlineStr"/>
+      <c r="L22" s="13" t="inlineStr"/>
+      <c r="M22" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O22" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>acrossai-mcp-manager</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>AcrossAI MCP Manager – WordPress MCP Server &amp; Admin for MCP Adapter, Claude &amp; ChatGPT</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>0.4.3</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>35</v>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H23" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="J23" s="24" t="inlineStr"/>
+      <c r="K23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>users, blocks</t>
+        </is>
+      </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O23" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>sokket-site-connector-for-mcp</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Sokket – MCP Server: Connect Claude, ChatGPT, Cursor &amp; Any AI Agent to WordPress</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G24" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H24" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="J24" s="24" t="inlineStr"/>
+      <c r="K24" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, plugins, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M24" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required. Provide a bearer token or an Application Password.)</t>
+        </is>
+      </c>
+      <c r="O24" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>webo-mcp</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>WEBO MCP</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>3.0.32</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>33</v>
+      </c>
+      <c r="J25" s="24" t="inlineStr"/>
+      <c r="K25" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>media, taxonomies, users, blocks</t>
+        </is>
+      </c>
+      <c r="M25" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O25" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>alphabridge-mcp</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>AlphaBridge MCP – Connect Claude and ChatGPT to WordPress</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>4.6.5</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G26" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H26" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="J26" s="24" t="inlineStr"/>
+      <c r="K26" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, users, settings</t>
+        </is>
+      </c>
+      <c r="M26" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N26" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Invalid or missing bearer token. Send the connection's token as "Authorization: Bearer …" or connect again; an administrator manages connections under Settings → AlphaBridge MCP.)</t>
+        </is>
+      </c>
+      <c r="O26" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>track-debug</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Track Debug – WordPress MCP Server: Connect Claude, ChatGPT &amp; AI Agents</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H27" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" s="24" t="inlineStr"/>
+      <c r="K27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="13" t="inlineStr"/>
+      <c r="M27" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N27" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O27" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>admindra-mcp</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>AdMindra MCP – AI Connector for ChatGPT &amp; Claude</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>1.1.2</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H28" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I28" s="24" t="inlineStr"/>
+      <c r="J28" s="24" t="inlineStr"/>
+      <c r="K28" s="24" t="inlineStr"/>
+      <c r="L28" s="13" t="inlineStr"/>
+      <c r="M28" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (MCP authentication required.)</t>
+        </is>
+      </c>
+      <c r="O28" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>devcubic-ai-bridge-for-mcp</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>DevCubic AI Bridge for MCP</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>1.0.3</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H29" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I29" s="24" t="inlineStr"/>
+      <c r="J29" s="24" t="inlineStr"/>
+      <c r="K29" s="24" t="inlineStr"/>
+      <c r="L29" s="13" t="inlineStr"/>
+      <c r="M29" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N29" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (A valid access token is required.)</t>
+        </is>
+      </c>
+      <c r="O29" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>abilities-bridge</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Abilities Bridge</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H30" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="24" t="inlineStr"/>
+      <c r="K30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="13" t="inlineStr"/>
+      <c r="M30" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required. Use OAuth Bearer token or WordPress Application Password.)</t>
+        </is>
+      </c>
+      <c r="O30" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>strifebridge-mcp</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>StrifeBridge MCP</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G31" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H31" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>34</v>
+      </c>
+      <c r="J31" s="24" t="inlineStr"/>
+      <c r="K31" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, plugins, settings</t>
+        </is>
+      </c>
+      <c r="M31" s="25" t="inlineStr">
+        <is>
+          <t>registers-abilities</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O31" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>bcs-mcp-manager</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>ByteCoreStack – MCP Connector for AI Tools</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>1.2.5</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G32" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H32" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I32" s="24" t="inlineStr"/>
+      <c r="J32" s="24" t="inlineStr"/>
+      <c r="K32" s="24" t="inlineStr"/>
+      <c r="L32" s="13" t="inlineStr"/>
+      <c r="M32" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N32" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Authentication required.)</t>
+        </is>
+      </c>
+      <c r="O32" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>saddle</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Saddle – AI Site Control (MCP)</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>1.5.2</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G33" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H33" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>41</v>
+      </c>
+      <c r="J33" s="24" t="inlineStr"/>
+      <c r="K33" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L33" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, users, settings, blocks</t>
+        </is>
+      </c>
+      <c r="M33" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N33" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O33" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>acadium-agent-publisher</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Acadium AI Site Editor</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>2.0.0</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G34" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="J34" s="24" t="inlineStr"/>
+      <c r="K34" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies</t>
+        </is>
+      </c>
+      <c r="M34" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N34" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O34" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>aicom</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>AICOM – AI Commander</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>3.22.2</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>API key</t>
+        </is>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>93</v>
+      </c>
+      <c r="J35" s="24" t="inlineStr"/>
+      <c r="K35" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L35" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, users, plugins, settings</t>
+        </is>
+      </c>
+      <c r="M35" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N35" s="13" t="inlineStr">
+        <is>
+          <t>initialize 200, tools/list 200 (API key missing)</t>
+        </is>
+      </c>
+      <c r="O35" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>rectus-content-access-for-mcp</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Rectus Content Access for MCP</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>1.7.2</t>
+        </is>
+      </c>
+      <c r="D36" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" s="24" t="n">
+        <v>68</v>
+      </c>
+      <c r="K36" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, media, taxonomies, blocks</t>
+        </is>
+      </c>
+      <c r="M36" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N36" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Sorry, you are not allowed to do that.)</t>
+        </is>
+      </c>
+      <c r="O36" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>mcp-for-woocommerce</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>MCP for WooCommerce</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>Public by design</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="J37" s="24" t="inlineStr"/>
+      <c r="K37" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L37" s="13" t="inlineStr">
+        <is>
+          <t>posts, pages, taxonomies, woocommerce</t>
+        </is>
+      </c>
+      <c r="M37" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N37" s="13" t="inlineStr">
+        <is>
+          <t>initialize 200, tools/list 200, 31 tools. Evidence: includes/Core/McpStreamableTransport.php:58-61: permission_callback __return_true, commented 'Intentionally public: every tool returns only storefront data a visitor can already see, nothing is written'</t>
+        </is>
+      </c>
+      <c r="O37" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>counterhand-mcp-for-woocommerce</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Counterhand MCP for WooCommerce — AI Agent Server for Claude, ChatGPT &amp; Cursor</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="I38" s="24" t="inlineStr"/>
+      <c r="J38" s="24" t="inlineStr"/>
+      <c r="K38" s="24" t="inlineStr"/>
+      <c r="L38" s="13" t="inlineStr"/>
+      <c r="M38" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N38" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401 (Invalid or missing API token.)</t>
+        </is>
+      </c>
+      <c r="O38" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>publishio</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Publishio – Build Pages &amp; Posts with ChatGPT and Claude using MCP</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>App password</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="J39" s="24" t="inlineStr"/>
+      <c r="K39" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" s="13" t="inlineStr">
+        <is>
+          <t>posts, media, taxonomies, blocks</t>
+        </is>
+      </c>
+      <c r="M39" s="25" t="inlineStr">
+        <is>
+          <t>mcp-adapter, reads-abilities, registers-abilities</t>
+        </is>
+      </c>
+      <c r="N39" s="13" t="inlineStr">
+        <is>
+          <t>initialize 401, tools/list 401</t>
+        </is>
+      </c>
+      <c r="O39" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G5:G39">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Y"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5144,13 +7710,13 @@
           <t>AI Engine – The Chatbot, AI Framework &amp; MCP for WordPress</t>
         </is>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="26" t="n">
         <v>90000</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="28">
         <f>Weights!$B$3-E5</f>
         <v/>
       </c>
@@ -5170,7 +7736,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/ai-engine/</t>
         </is>
@@ -5197,13 +7763,13 @@
           <t>WPVibe – MCP Server for WordPress, works with Claude, ChatGPT &amp; other AI MCP agents</t>
         </is>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="28">
         <f>Weights!$B$3-E6</f>
         <v/>
       </c>
@@ -5223,7 +7789,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K6" s="27" t="inlineStr">
+      <c r="K6" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/vibe-ai/</t>
         </is>
@@ -5250,13 +7816,13 @@
           <t>Easy MCP AI – Connect Claude to WordPress: MCP Server for ChatGPT &amp; AI Agents</t>
         </is>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="26" t="n">
         <v>20000</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="27" t="n">
         <v>46310</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="28">
         <f>Weights!$B$3-E7</f>
         <v/>
       </c>
@@ -5276,7 +7842,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K7" s="27" t="inlineStr">
+      <c r="K7" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/easy-mcp-ai/</t>
         </is>
@@ -5303,13 +7869,13 @@
           <t>Royal MCP – Secure AI Connector for Claude, ChatGPT &amp; any LLM via MCP</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="26" t="n">
         <v>10000</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="27" t="n">
         <v>46310</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="28">
         <f>Weights!$B$3-E8</f>
         <v/>
       </c>
@@ -5329,7 +7895,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K8" s="27" t="inlineStr">
+      <c r="K8" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/royal-mcp/</t>
         </is>
@@ -5356,13 +7922,13 @@
           <t>Secure MCP Server for Claude, ChatGPT, Gemini and other AI Agents</t>
         </is>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="26" t="n">
         <v>6000</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="27" t="n">
         <v>46303</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="28">
         <f>Weights!$B$3-E9</f>
         <v/>
       </c>
@@ -5382,7 +7948,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K9" s="27" t="inlineStr">
+      <c r="K9" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/miniorange-secure-mcp-server/</t>
         </is>
@@ -5409,13 +7975,13 @@
           <t>WSP MCP – Free MCP Plugin for WordPress: Connect Claude, ChatGPT &amp; AI Agents</t>
         </is>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="26" t="n">
         <v>2000</v>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="27" t="n">
         <v>46308</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="28">
         <f>Weights!$B$3-E10</f>
         <v/>
       </c>
@@ -5435,7 +8001,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K10" s="27" t="inlineStr">
+      <c r="K10" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/wsp-mcp-ai-agents-connector/</t>
         </is>
@@ -5462,13 +8028,13 @@
           <t>Cowboy MCP – Free MCP Server with Undo for Claude &amp; ChatGPT</t>
         </is>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="26" t="n">
         <v>1000</v>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="28">
         <f>Weights!$B$3-E11</f>
         <v/>
       </c>
@@ -5488,7 +8054,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K11" s="27" t="inlineStr">
+      <c r="K11" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/cowboy-mcp/</t>
         </is>
@@ -5515,13 +8081,13 @@
           <t>Flex MCP – Connect ChatGPT, Claude and AI agents with MCP, Undo, Abilities and Tools.</t>
         </is>
       </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="26" t="n">
         <v>800</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="27" t="n">
         <v>46308</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="28">
         <f>Weights!$B$3-E12</f>
         <v/>
       </c>
@@ -5541,7 +8107,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K12" s="27" t="inlineStr">
+      <c r="K12" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/stifli-flex-mcp/</t>
         </is>
@@ -5568,13 +8134,13 @@
           <t>Agent Abilities for MCP – Connect Claude and ChatGPT with Permission Controls and Audit Log</t>
         </is>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="26" t="n">
         <v>600</v>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="27" t="n">
         <v>46310</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="28">
         <f>Weights!$B$3-E13</f>
         <v/>
       </c>
@@ -5594,7 +8160,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K13" s="27" t="inlineStr">
+      <c r="K13" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/agent-abilities-for-mcp/</t>
         </is>
@@ -5621,13 +8187,13 @@
           <t>DiviOps Agent</t>
         </is>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="26" t="n">
         <v>500</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="28">
         <f>Weights!$B$3-E14</f>
         <v/>
       </c>
@@ -5647,7 +8213,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K14" s="27" t="inlineStr">
+      <c r="K14" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/diviops-agent/</t>
         </is>
@@ -5674,13 +8240,13 @@
           <t>MCP Server for WordPress – Connect Claude, ChatGPT &amp; Gemini | AtlasMCP</t>
         </is>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="26" t="n">
         <v>300</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E15" s="27" t="n">
         <v>46304</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="28">
         <f>Weights!$B$3-E15</f>
         <v/>
       </c>
@@ -5700,7 +8266,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K15" s="27" t="inlineStr">
+      <c r="K15" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/ai-workflow-automation-ai-agent-hub/</t>
         </is>
@@ -5727,13 +8293,13 @@
           <t>NIBWP – Self-Hosted MCP Server – Connect Claude, ChatGPT, Cursor &amp; Any AI Agent via MCP</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="26" t="n">
         <v>300</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="27" t="n">
         <v>46295</v>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="28">
         <f>Weights!$B$3-E16</f>
         <v/>
       </c>
@@ -5753,7 +8319,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K16" s="27" t="inlineStr">
+      <c r="K16" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/nibwp/</t>
         </is>
@@ -5780,13 +8346,13 @@
           <t>MountDev AI MCP Connector for WordPress</t>
         </is>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="26" t="n">
         <v>200</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="27" t="n">
         <v>46296</v>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="28">
         <f>Weights!$B$3-E17</f>
         <v/>
       </c>
@@ -5806,7 +8372,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K17" s="27" t="inlineStr">
+      <c r="K17" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/mountdev-ai-mcp-connector/</t>
         </is>
@@ -5833,13 +8399,13 @@
           <t>IATO MCP</t>
         </is>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="E18" s="25" t="n">
+      <c r="E18" s="27" t="n">
         <v>46310</v>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="28">
         <f>Weights!$B$3-E18</f>
         <v/>
       </c>
@@ -5859,7 +8425,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K18" s="27" t="inlineStr">
+      <c r="K18" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/iato-mcp/</t>
         </is>
@@ -5886,13 +8452,13 @@
           <t>SiteSkite – Secure MCP &amp; AI WebOps. Connect ChatGPT, Claude, or Any AI Agent via MCP</t>
         </is>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="E19" s="27" t="n">
         <v>46305</v>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="28">
         <f>Weights!$B$3-E19</f>
         <v/>
       </c>
@@ -5912,7 +8478,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K19" s="27" t="inlineStr">
+      <c r="K19" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/siteskite/</t>
         </is>
@@ -5939,13 +8505,13 @@
           <t>Invizo MCP – Secure AI Connector for Claude, Codex, Cursor and WooCommerce</t>
         </is>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="E20" s="25" t="n">
+      <c r="E20" s="27" t="n">
         <v>46222</v>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="28">
         <f>Weights!$B$3-E20</f>
         <v/>
       </c>
@@ -5965,7 +8531,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K20" s="27" t="inlineStr">
+      <c r="K20" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/invizo-mcp/</t>
         </is>
@@ -5992,13 +8558,13 @@
           <t>YLabs AI Assistant Connector</t>
         </is>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="26" t="n">
         <v>1000</v>
       </c>
-      <c r="E21" s="25" t="n">
+      <c r="E21" s="27" t="n">
         <v>46274</v>
       </c>
-      <c r="F21" s="26">
+      <c r="F21" s="28">
         <f>Weights!$B$3-E21</f>
         <v/>
       </c>
@@ -6018,7 +8584,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K21" s="27" t="inlineStr">
+      <c r="K21" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/ylabs-ai-assistant-connector/</t>
         </is>
@@ -6045,13 +8611,13 @@
           <t>Albert – Connect AI Assistants to WordPress</t>
         </is>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E22" s="27" t="n">
         <v>46290</v>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="28">
         <f>Weights!$B$3-E22</f>
         <v/>
       </c>
@@ -6071,7 +8637,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K22" s="27" t="inlineStr">
+      <c r="K22" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/albert-ai-butler/</t>
         </is>
@@ -6098,13 +8664,13 @@
           <t>AcrossAI MCP Manager – WordPress MCP Server &amp; Admin for MCP Adapter, Claude &amp; ChatGPT</t>
         </is>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="26" t="n">
         <v>40</v>
       </c>
-      <c r="E23" s="25" t="n">
+      <c r="E23" s="27" t="n">
         <v>46303</v>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="28">
         <f>Weights!$B$3-E23</f>
         <v/>
       </c>
@@ -6124,7 +8690,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K23" s="27" t="inlineStr">
+      <c r="K23" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/acrossai-mcp-manager/</t>
         </is>
@@ -6151,13 +8717,13 @@
           <t>Sokket – MCP Server: Connect Claude, ChatGPT, Cursor &amp; Any AI Agent to WordPress</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n">
+      <c r="D24" s="26" t="n">
         <v>70</v>
       </c>
-      <c r="E24" s="25" t="n">
+      <c r="E24" s="27" t="n">
         <v>46296</v>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="28">
         <f>Weights!$B$3-E24</f>
         <v/>
       </c>
@@ -6177,7 +8743,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K24" s="27" t="inlineStr">
+      <c r="K24" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/sokket-site-connector-for-mcp/</t>
         </is>
@@ -6204,13 +8770,13 @@
           <t>WEBO MCP</t>
         </is>
       </c>
-      <c r="D25" s="24" t="n">
+      <c r="D25" s="26" t="n">
         <v>40</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="27" t="n">
         <v>46291</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="28">
         <f>Weights!$B$3-E25</f>
         <v/>
       </c>
@@ -6230,7 +8796,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K25" s="27" t="inlineStr">
+      <c r="K25" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/webo-mcp/</t>
         </is>
@@ -6257,13 +8823,13 @@
           <t>AlphaBridge MCP – Connect Claude and ChatGPT to WordPress</t>
         </is>
       </c>
-      <c r="D26" s="24" t="n">
+      <c r="D26" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="E26" s="25" t="n">
+      <c r="E26" s="27" t="n">
         <v>46307</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="28">
         <f>Weights!$B$3-E26</f>
         <v/>
       </c>
@@ -6283,7 +8849,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K26" s="27" t="inlineStr">
+      <c r="K26" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/alphabridge-mcp/</t>
         </is>
@@ -6310,13 +8876,13 @@
           <t>Track Debug – WordPress MCP Server: Connect Claude, ChatGPT &amp; AI Agents</t>
         </is>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="27" t="n">
         <v>46306</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="28">
         <f>Weights!$B$3-E27</f>
         <v/>
       </c>
@@ -6336,7 +8902,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K27" s="27" t="inlineStr">
+      <c r="K27" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/track-debug/</t>
         </is>
@@ -6363,13 +8929,13 @@
           <t>AdMindra MCP – AI Connector for ChatGPT &amp; Claude</t>
         </is>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="25" t="n">
+      <c r="E28" s="27" t="n">
         <v>46306</v>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="28">
         <f>Weights!$B$3-E28</f>
         <v/>
       </c>
@@ -6389,7 +8955,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K28" s="27" t="inlineStr">
+      <c r="K28" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/admindra-mcp/</t>
         </is>
@@ -6416,13 +8982,13 @@
           <t>DevCubic AI Bridge for MCP</t>
         </is>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="25" t="n">
+      <c r="E29" s="27" t="n">
         <v>46309</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="28">
         <f>Weights!$B$3-E29</f>
         <v/>
       </c>
@@ -6442,7 +9008,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K29" s="27" t="inlineStr">
+      <c r="K29" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/devcubic-ai-bridge-for-mcp/</t>
         </is>
@@ -6469,13 +9035,13 @@
           <t>Abilities Bridge</t>
         </is>
       </c>
-      <c r="D30" s="24" t="n">
+      <c r="D30" s="26" t="n">
         <v>80</v>
       </c>
-      <c r="E30" s="25" t="n">
+      <c r="E30" s="27" t="n">
         <v>46286</v>
       </c>
-      <c r="F30" s="26">
+      <c r="F30" s="28">
         <f>Weights!$B$3-E30</f>
         <v/>
       </c>
@@ -6495,7 +9061,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K30" s="27" t="inlineStr">
+      <c r="K30" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/abilities-bridge/</t>
         </is>
@@ -6522,13 +9088,13 @@
           <t>StrifeBridge MCP</t>
         </is>
       </c>
-      <c r="D31" s="24" t="n">
+      <c r="D31" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="E31" s="25" t="n">
+      <c r="E31" s="27" t="n">
         <v>46267</v>
       </c>
-      <c r="F31" s="26">
+      <c r="F31" s="28">
         <f>Weights!$B$3-E31</f>
         <v/>
       </c>
@@ -6548,7 +9114,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K31" s="27" t="inlineStr">
+      <c r="K31" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/strifebridge-mcp/</t>
         </is>
@@ -6575,13 +9141,13 @@
           <t>ByteCoreStack – MCP Connector for AI Tools</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n">
+      <c r="D32" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="E32" s="25" t="n">
+      <c r="E32" s="27" t="n">
         <v>46289</v>
       </c>
-      <c r="F32" s="26">
+      <c r="F32" s="28">
         <f>Weights!$B$3-E32</f>
         <v/>
       </c>
@@ -6601,7 +9167,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K32" s="27" t="inlineStr">
+      <c r="K32" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/bcs-mcp-manager/</t>
         </is>
@@ -6628,13 +9194,13 @@
           <t>Saddle – AI Site Control (MCP)</t>
         </is>
       </c>
-      <c r="D33" s="24" t="n">
+      <c r="D33" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="E33" s="25" t="n">
+      <c r="E33" s="27" t="n">
         <v>46307</v>
       </c>
-      <c r="F33" s="26">
+      <c r="F33" s="28">
         <f>Weights!$B$3-E33</f>
         <v/>
       </c>
@@ -6654,7 +9220,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K33" s="27" t="inlineStr">
+      <c r="K33" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/saddle/</t>
         </is>
@@ -6681,13 +9247,13 @@
           <t>Acadium AI Site Editor</t>
         </is>
       </c>
-      <c r="D34" s="24" t="n">
+      <c r="D34" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="25" t="n">
+      <c r="E34" s="27" t="n">
         <v>46303</v>
       </c>
-      <c r="F34" s="26">
+      <c r="F34" s="28">
         <f>Weights!$B$3-E34</f>
         <v/>
       </c>
@@ -6707,7 +9273,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K34" s="27" t="inlineStr">
+      <c r="K34" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/acadium-agent-publisher/</t>
         </is>
@@ -6734,13 +9300,13 @@
           <t>AICOM – AI Commander</t>
         </is>
       </c>
-      <c r="D35" s="24" t="n">
+      <c r="D35" s="26" t="n">
         <v>60</v>
       </c>
-      <c r="E35" s="25" t="n">
+      <c r="E35" s="27" t="n">
         <v>46308</v>
       </c>
-      <c r="F35" s="26">
+      <c r="F35" s="28">
         <f>Weights!$B$3-E35</f>
         <v/>
       </c>
@@ -6760,7 +9326,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K35" s="27" t="inlineStr">
+      <c r="K35" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/aicom/</t>
         </is>
@@ -6787,13 +9353,13 @@
           <t>Rectus Content Access for MCP</t>
         </is>
       </c>
-      <c r="D36" s="24" t="n">
+      <c r="D36" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="25" t="n">
+      <c r="E36" s="27" t="n">
         <v>46301</v>
       </c>
-      <c r="F36" s="26">
+      <c r="F36" s="28">
         <f>Weights!$B$3-E36</f>
         <v/>
       </c>
@@ -6813,7 +9379,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K36" s="27" t="inlineStr">
+      <c r="K36" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/rectus-content-access-for-mcp/</t>
         </is>
@@ -6840,13 +9406,13 @@
           <t>MCP for WooCommerce</t>
         </is>
       </c>
-      <c r="D37" s="24" t="n">
+      <c r="D37" s="26" t="n">
         <v>60</v>
       </c>
-      <c r="E37" s="25" t="n">
+      <c r="E37" s="27" t="n">
         <v>46302</v>
       </c>
-      <c r="F37" s="26">
+      <c r="F37" s="28">
         <f>Weights!$B$3-E37</f>
         <v/>
       </c>
@@ -6866,7 +9432,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K37" s="27" t="inlineStr">
+      <c r="K37" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/mcp-for-woocommerce/</t>
         </is>
@@ -6893,13 +9459,13 @@
           <t>Counterhand MCP for WooCommerce — AI Agent Server for Claude, ChatGPT &amp; Cursor</t>
         </is>
       </c>
-      <c r="D38" s="24" t="n">
+      <c r="D38" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="E38" s="25" t="n">
+      <c r="E38" s="27" t="n">
         <v>46308</v>
       </c>
-      <c r="F38" s="26">
+      <c r="F38" s="28">
         <f>Weights!$B$3-E38</f>
         <v/>
       </c>
@@ -6919,7 +9485,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K38" s="27" t="inlineStr">
+      <c r="K38" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/counterhand-mcp-for-woocommerce/</t>
         </is>
@@ -6946,13 +9512,13 @@
           <t>Publishio – Build Pages &amp; Posts with ChatGPT and Claude using MCP</t>
         </is>
       </c>
-      <c r="D39" s="24" t="n">
+      <c r="D39" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="E39" s="25" t="n">
+      <c r="E39" s="27" t="n">
         <v>46279</v>
       </c>
-      <c r="F39" s="26">
+      <c r="F39" s="28">
         <f>Weights!$B$3-E39</f>
         <v/>
       </c>
@@ -6972,7 +9538,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K39" s="27" t="inlineStr">
+      <c r="K39" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/publishio/</t>
         </is>
@@ -6999,13 +9565,13 @@
           <t>MCP Adapter</t>
         </is>
       </c>
-      <c r="D40" s="24" t="n">
+      <c r="D40" s="26" t="n">
         <v>40000</v>
       </c>
-      <c r="E40" s="25" t="n">
+      <c r="E40" s="27" t="n">
         <v>46297</v>
       </c>
-      <c r="F40" s="26">
+      <c r="F40" s="28">
         <f>Weights!$B$3-E40</f>
         <v/>
       </c>
@@ -7025,7 +9591,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K40" s="27" t="inlineStr">
+      <c r="K40" s="29" t="inlineStr">
         <is>
           <t>https://wordpress.org/plugins/mcp-adapter/</t>
         </is>
@@ -7079,7 +9645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7101,12 +9667,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>Data as of</t>
         </is>
       </c>
-      <c r="B3" s="29" t="n">
+      <c r="B3" s="31" t="n">
         <v>46310</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -7116,9 +9682,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="n"/>
-      <c r="B4" s="28" t="n"/>
-      <c r="C4" s="28" t="n"/>
+      <c r="A4" s="30" t="n"/>
+      <c r="B4" s="30" t="n"/>
+      <c r="C4" s="30" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -7131,88 +9697,88 @@
           <t>Weight</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n"/>
+      <c r="C5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Setup &amp; connection</t>
         </is>
       </c>
-      <c r="B6" s="30" t="n">
+      <c r="B6" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="C6" s="28" t="n"/>
+      <c r="C6" s="30" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Security &amp; auth</t>
         </is>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="C7" s="28" t="n"/>
+      <c r="C7" s="30" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Capabilities</t>
         </is>
       </c>
-      <c r="B8" s="30" t="n">
+      <c r="B8" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="28" t="n"/>
+      <c r="C8" s="30" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Quality &amp; maintenance</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="C9" s="28" t="n"/>
+      <c r="C9" s="30" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="33">
         <f>SUM(B6:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="30">
         <f>IF(B10=100,"OK","Weights must total 100")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="n"/>
-      <c r="B11" s="28" t="n"/>
-      <c r="C11" s="28" t="n"/>
+      <c r="A11" s="30" t="n"/>
+      <c r="B11" s="30" t="n"/>
+      <c r="C11" s="30" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Security hard-fail cap</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n"/>
-      <c r="C12" s="28" t="n"/>
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="30" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Max total score if 'Security hard fail?' = Y</t>
         </is>
       </c>
-      <c r="B13" s="30" t="n">
+      <c r="B13" s="32" t="n">
         <v>40</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -7222,120 +9788,120 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="n"/>
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="28" t="n"/>
+      <c r="A14" s="30" t="n"/>
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="30" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>Update recency thresholds (days since last update, for 5 / 4 / 3 / 2 points; older = 1)</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n"/>
-      <c r="C15" s="28" t="n"/>
+      <c r="B15" s="30" t="n"/>
+      <c r="C15" s="30" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>5 points if updated within (days)</t>
         </is>
       </c>
-      <c r="B16" s="30" t="n">
+      <c r="B16" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="C16" s="28" t="n"/>
+      <c r="C16" s="30" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>4 points if updated within (days)</t>
         </is>
       </c>
-      <c r="B17" s="30" t="n">
+      <c r="B17" s="32" t="n">
         <v>90</v>
       </c>
-      <c r="C17" s="28" t="n"/>
+      <c r="C17" s="30" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>3 points if updated within (days)</t>
         </is>
       </c>
-      <c r="B18" s="30" t="n">
+      <c r="B18" s="32" t="n">
         <v>180</v>
       </c>
-      <c r="C18" s="28" t="n"/>
+      <c r="C18" s="30" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>2 points if updated within (days)</t>
         </is>
       </c>
-      <c r="B19" s="30" t="n">
+      <c r="B19" s="32" t="n">
         <v>365</v>
       </c>
-      <c r="C19" s="28" t="n"/>
+      <c r="C19" s="30" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="n"/>
-      <c r="B20" s="28" t="n"/>
-      <c r="C20" s="28" t="n"/>
+      <c r="A20" s="30" t="n"/>
+      <c r="B20" s="30" t="n"/>
+      <c r="C20" s="30" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>Adoption thresholds (active installs, for 5 / 4 / 3 / 2 points; fewer = 1)</t>
         </is>
       </c>
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="28" t="n"/>
+      <c r="B21" s="30" t="n"/>
+      <c r="C21" s="30" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>5 points if installs at least</t>
         </is>
       </c>
-      <c r="B22" s="32" t="n">
+      <c r="B22" s="34" t="n">
         <v>10000</v>
       </c>
-      <c r="C22" s="28" t="n"/>
+      <c r="C22" s="30" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>4 points if installs at least</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="C23" s="28" t="n"/>
+      <c r="C23" s="30" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>3 points if installs at least</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="C24" s="28" t="n"/>
+      <c r="C24" s="30" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>2 points if installs at least</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="C25" s="28" t="n"/>
+      <c r="C25" s="30" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">

</xml_diff>